<commit_message>
S3 : exercices + mini projet S1 --> S3
</commit_message>
<xml_diff>
--- a/Projets/01 Parcours Data Engineer/Planning_Data_Engineer.xlsx
+++ b/Projets/01 Parcours Data Engineer/Planning_Data_Engineer.xlsx
@@ -706,12 +706,12 @@
       </c>
       <c r="I6" s="16" t="inlineStr">
         <is>
-          <t>En cours</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>Démarrée le 29/06 : fiche pandas fondamentaux + exercice s2_1.</t>
+          <t>Livrable analyse exploratoire fait. Clôturée.</t>
         </is>
       </c>
     </row>
@@ -756,10 +756,14 @@
       </c>
       <c r="I7" s="16" t="inlineStr">
         <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="J7" s="14" t="n"/>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>Cours (groupby, window functions, OOP) + exercices + mini-projet cumulatif S1-&gt;S3 faits. À pousser sur GitHub.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="87.75" customHeight="1">
       <c r="A8" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Refactorisation de la structure des CLAUDE.md (méthode générique et spécifique DE) et finalisation de la S7 (exercices Java/Spark et mise à jour des fiches).
</commit_message>
<xml_diff>
--- a/Projets/01 Parcours Data Engineer/Planning_Data_Engineer.xlsx
+++ b/Projets/01 Parcours Data Engineer/Planning_Data_Engineer.xlsx
@@ -806,10 +806,14 @@
       </c>
       <c r="I8" s="16" t="inlineStr">
         <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="J8" s="14" t="n"/>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>Pandas avancé (merge/concat, pivot_table, apply) + SQL CTE + API-&gt;pandas + mini-projet cumulatif S1-&gt;S4. Poussé sur GitHub.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="87.75" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -852,10 +856,14 @@
       </c>
       <c r="I9" s="16" t="inlineStr">
         <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="n"/>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>Projet ETL 1 (projet-01-etl) : extract CSV+JSON, transform pandas, load PostgreSQL via SQLAlchemy, .env, logging. Sur GitHub.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="87.75" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
@@ -898,10 +906,14 @@
       </c>
       <c r="I10" s="16" t="inlineStr">
         <is>
-          <t>À faire</t>
-        </is>
-      </c>
-      <c r="J10" s="14" t="n"/>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>Concepts DE (ETL/ELT, batch/streaming, warehouse/lake, idempotence), modélisation en étoile, Airflow. Exercices écrits. Sur GitHub.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="87.75" customHeight="1">
       <c r="A11" s="10" t="inlineStr">

</xml_diff>